<commit_message>
brs pre-tweaks, SPR competitor without deviation decrease
</commit_message>
<xml_diff>
--- a/changes/fal-stocks.xlsx
+++ b/changes/fal-stocks.xlsx
@@ -497,6 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <dimension ref="A1:N41"/>
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
@@ -952,16 +953,24 @@
       <c r="B18" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="4">
-        <v>2.0</v>
-      </c>
-      <c r="D18" s="4">
-        <v>0.08</v>
+      <c r="C18" t="inlineStr" s="4">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr" s="4">
+        <is>
+          <t>0.05</t>
+        </is>
       </c>
       <c r="E18" s="4">
         <v>-1.0</v>
       </c>
-      <c r="F18" s="4"/>
+      <c r="F18" t="inlineStr" s="4">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -1015,8 +1024,10 @@
       <c r="B20" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="4">
-        <v>8.0</v>
+      <c r="C20" t="inlineStr" s="4">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="D20" s="4">
         <v>0.23</v>
@@ -1024,8 +1035,10 @@
       <c r="E20" s="4">
         <v>-10.0</v>
       </c>
-      <c r="F20" s="4">
-        <v>-10.0</v>
+      <c r="F20" t="inlineStr" s="4">
+        <is>
+          <t>-8</t>
+        </is>
       </c>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
@@ -1046,8 +1059,10 @@
       <c r="B21" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="4">
-        <v>5.0</v>
+      <c r="C21" t="inlineStr" s="4">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="D21" s="4">
         <v>0.12</v>

</xml_diff>